<commit_message>
Drop outreach_locations column (only 5 of 115 offices had values)
</commit_message>
<xml_diff>
--- a/data/processed/services_structured.xlsx
+++ b/data/processed/services_structured.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Referents" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offices'!$A$1:$Q$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offices'!$A$1:$P$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Services'!$A$1:$G$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Coverage'!$A$1:$J$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Referents'!$A$1:$F$14</definedName>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q116"/>
+  <dimension ref="A1:P116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -447,13 +447,12 @@
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="50" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,35 +508,30 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>outreach_locations</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>email</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>website</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>source_url</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>source_url</t>
+          <t>filled_fields</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>filled_fields</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>is_caritas</t>
         </is>
@@ -596,35 +590,30 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66659</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0931 386-66659</t>
+          <t>martina.zawierta@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>martina.zawierta@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/kuren-und-erholung/</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/kuren-und-erholung/</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q2" t="b">
+      <c r="P2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -681,35 +670,30 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66662</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0931 386-66662</t>
+          <t>heike.korbmann@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>heike.korbmann@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/kuren-und-erholung/</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/kuren-und-erholung/</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q3" t="b">
+      <c r="P3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -766,17 +750,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 392-301</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>06021 392-301</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -786,15 +770,10 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
           <t>organisation, website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q4" t="b">
+      <c r="P4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -851,17 +830,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0971 7246-9200</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0971 7246-9200</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -871,15 +850,10 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
           <t>organisation, website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q5" t="b">
+      <c r="P5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -936,17 +910,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Mellrichstadt  Bad Königshofen</t>
+          <t>09771 6116-15</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>09771 6116-15</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -956,15 +930,10 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
           <t>website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q6" t="b">
+      <c r="P6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1021,17 +990,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Ebern - Graf-Stauffenberg-Str. 19a</t>
+          <t>09521 69131</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>09521 69131</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1041,15 +1010,10 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
           <t>website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q7" t="b">
+      <c r="P7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1106,17 +1070,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Stadtteilzentrum Kitzingen, Volkach</t>
+          <t>09321 7817</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>09321 7817</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1126,15 +1090,10 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
           <t>website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q8" t="b">
+      <c r="P8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1191,17 +1150,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Elsenfeld - Hofstetter Straße 3</t>
+          <t>09371 9789-20</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>09371 9789-20</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1211,15 +1170,10 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
           <t>website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q9" t="b">
+      <c r="P9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1276,17 +1230,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Giebelstadt - Obere Kirchgasse 6 - 09334 993242  Ochsenfurt - Kellereistraße 8 - 0931 804570</t>
+          <t>0931 4190461</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0931 4190461</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1296,15 +1250,10 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/erziehungshilfe/</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
           <t>website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q10" t="b">
+      <c r="P10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1361,35 +1310,30 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09385/81 10</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>09385/81 10</t>
+          <t>t.buchner@antonia-werr-zentrum.de</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>t.buchner@antonia-werr-zentrum.de</t>
+          <t>https://www.antonia-werr-zentrum.de</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.antonia-werr-zentrum.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q11" t="b">
+      <c r="P11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1446,35 +1390,30 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/41 92-167</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0931/41 92-167</t>
+          <t>glemnitz@bbw-wuerzburg.de</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>glemnitz@bbw-wuerzburg.de</t>
+          <t>https://www.bbw-wuerzburg.de</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.bbw-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q12" t="b">
+      <c r="P12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1531,35 +1470,30 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/41 92-605</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0931/41 92-605</t>
+          <t>hitz@bbw-wuerzburg.de</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>hitz@bbw-wuerzburg.de</t>
+          <t>https://www.bbw-wuerzburg.de</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.bbw-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q13" t="b">
+      <c r="P13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1616,35 +1550,30 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 / 3046940</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0931 / 3046940</t>
+          <t>schulsozialarbeit@dbs-wuerzburg.de</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>schulsozialarbeit@dbs-wuerzburg.de</t>
+          <t>https://www.dbs-wuerzburg.de</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://www.dbs-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q14" t="b">
+      <c r="P14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1701,35 +1630,30 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 / 3046940</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0931 / 3046940</t>
+          <t>kranert@dbs-wuerzburg.de</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>kranert@dbs-wuerzburg.de</t>
+          <t>https://www.dbs-wuerzburg.de</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.dbs-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q15" t="b">
+      <c r="P15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1786,35 +1710,30 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721/78 99-155</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>09721/78 99-155</t>
+          <t>gertrud.tuerk@gbf-sw.de</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>gertrud.tuerk@gbf-sw.de</t>
+          <t>https://www.gbf-sw.de</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.gbf-sw.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q16" t="b">
+      <c r="P16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1871,35 +1790,30 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06024/67 34-13</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>06024/67 34-13</t>
+          <t>Bereichsleitung-BvB@haus-mirjam.de</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Bereichsleitung-BvB@haus-mirjam.de</t>
+          <t>https://www.haus-mirjam.de</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.haus-mirjam.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q17" t="b">
+      <c r="P17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1956,35 +1870,30 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/386 66-820</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0931/386 66-820</t>
+          <t>martina.fallmann@invia-wuerzburg.de</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>martina.fallmann@invia-wuerzburg.de</t>
+          <t>https://www.invia-wuerzburg.de</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.invia-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q18" t="b">
+      <c r="P18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2041,35 +1950,30 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/46 07 95 10</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0931/46 07 95 10</t>
+          <t>dick.bernadette@skf-wue.de</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>dick.bernadette@skf-wue.de</t>
+          <t>https://www.skf-wue.de</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://www.skf-wue.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
           <t>organisation, website</t>
         </is>
       </c>
-      <c r="Q19" t="b">
+      <c r="P19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2126,35 +2030,30 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721/78 83-270</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>09721/78 83-270</t>
+          <t>maria.kraft@kolping-mainfranken.de</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>maria.kraft@kolping-mainfranken.de</t>
+          <t>https://www.kolping-mainfranken.de</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.kolping-mainfranken.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q20" t="b">
+      <c r="P20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2211,35 +2110,30 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/600 84-0</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0931/600 84-0</t>
+          <t>christine.fabri@kolping-mainfranken.de</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>christine.fabri@kolping-mainfranken.de</t>
+          <t>https://www.kolping-mainfranken.de</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://www.kolping-mainfranken.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q21" t="b">
+      <c r="P21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2296,35 +2190,30 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/41 999-513</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0931/41 999-513</t>
+          <t>manfred.eck@kolping-mainfranken.de</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>manfred.eck@kolping-mainfranken.de</t>
+          <t>https://www.kolping-mainfranken.de</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://www.kolping-mainfranken.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q22" t="b">
+      <c r="P22" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2381,35 +2270,30 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/43 055</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0931/43 055</t>
+          <t>egner@dbs-wuerzburg.de</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>egner@dbs-wuerzburg.de</t>
+          <t>http://www.dbs-wuerzburg.de</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>http://www.dbs-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Q23" t="b">
+      <c r="P23" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2466,17 +2350,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931/386 58-607</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0931/386 58-607</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2486,15 +2370,10 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendsozialarbeit/</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
           <t>website, contact_person, email</t>
         </is>
       </c>
-      <c r="Q24" t="b">
+      <c r="P24" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2551,35 +2430,30 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0971 72469203</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0971 72469203</t>
+          <t>v.bartzsch@caritas-kissingen.de</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>v.bartzsch@caritas-kissingen.de</t>
+          <t>https://www.caritas-kissingen.de</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://www.caritas-kissingen.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/suchtberatung/</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q25" t="b">
+      <c r="P25" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2636,35 +2510,30 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 926563</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>09521 926563</t>
+          <t>jugendsuchtberatung@caritas-hassberge.de</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>jugendsuchtberatung@caritas-hassberge.de</t>
+          <t>https://www.caritas-hassberge.de</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://www.caritas-hassberge.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/suchtberatung/</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q26" t="b">
+      <c r="P26" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2721,35 +2590,30 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 59056</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0931 59056</t>
+          <t>mail@drogenberatung-wuerzburg.de</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>mail@drogenberatung-wuerzburg.de</t>
+          <t>http://www.drogenberatung-wuerzburg.de</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>http://www.drogenberatung-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/suchtberatung/</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q27" t="b">
+      <c r="P27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2806,35 +2670,30 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 38660-0</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>06021 38660-0</t>
+          <t>info@fruehfoerderung-aschaffenburg.de</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>info@fruehfoerderung-aschaffenburg.de</t>
+          <t>http://www.fruehfoerderung-aschaffenburg.de</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>http://www.fruehfoerderung-aschaffenburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q28" t="b">
+      <c r="P28" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2891,35 +2750,30 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09382 315484</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>09382 315484</t>
+          <t>info@fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>info@fruehfoerderstelle-geo.de</t>
+          <t>http://www.fruehforderstelle-geo.de</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>http://www.fruehforderstelle-geo.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q29" t="b">
+      <c r="P29" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2976,35 +2830,30 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 8776</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>09521 8776</t>
+          <t>info@fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>info@fruehfoerderstelle-geo.de</t>
+          <t>http://www.fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>http://www.fruehfoerderstelle-geo.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q30" t="b">
+      <c r="P30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3061,35 +2910,30 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09391 9188803</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>09391 9188803</t>
+          <t>info@fruehfoerderstelle.de</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>info@fruehfoerderstelle.de</t>
+          <t>https://www.fruehfoerderstelle.de</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://www.fruehfoerderstelle.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q31" t="b">
+      <c r="P31" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3146,35 +2990,30 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721 4741002</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>09721 4741002</t>
+          <t>info@fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>info@fruehfoerderstelle-geo.de</t>
+          <t>http://www.fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>http://www.fruehfoerderstelle-geo.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q32" t="b">
+      <c r="P32" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3231,35 +3070,30 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09382 315484</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>09382 315484</t>
+          <t>info@fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>info@fruehfoerderstelle-geo.de</t>
+          <t>http://www.fruehfoerderstelle-geo.de</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>http://www.fruehfoerderstelle-geo.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q33" t="b">
+      <c r="P33" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3316,17 +3150,17 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 8006-200</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0931 8006-200</t>
+          <t>maria-stern-schule@t-online.de</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>maria-stern-schule@t-online.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -3336,15 +3170,10 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q34" t="b">
+      <c r="P34" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3401,35 +3230,30 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 98081-0</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0931 98081-0</t>
+          <t>ff@fruehfoerderung-wuerzburg.de</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>ff@fruehfoerderung-wuerzburg.de</t>
+          <t>http://www.fruehfoerderung-wuerzburg.de</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>http://www.fruehfoerderung-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/fruehfoerderung/</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q35" t="b">
+      <c r="P35" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3486,35 +3310,30 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66659</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0931 386-66659</t>
+          <t>martina.zawierta@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>martina.zawierta@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/kur-und-erholung/</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/kinder/kur-und-erholung/</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q36" t="b">
+      <c r="P36" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3571,17 +3390,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3591,15 +3410,10 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
           <t>website, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q37" t="b">
+      <c r="P37" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3656,35 +3470,30 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 392-206</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>06021 392-206</t>
+          <t>info@caritas-aschaffenburg.de</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>info@caritas-aschaffenburg.de</t>
+          <t>https://www.caritas-aschaffenburg.de/sie-suchen-hilfe/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>https://www.caritas-aschaffenburg.de/sie-suchen-hilfe/allgemeine-sozialberatung/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q38" t="b">
+      <c r="P38" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3741,35 +3550,30 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0971 7246-17</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0971 7246-17</t>
+          <t>asbd@caritas-kissingen.de</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>asbd@caritas-kissingen.de</t>
+          <t>https://www.caritas-kissingen.de/beratung-und-hilfe/allgemeiner-sozialer-beratungsdienst</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>https://www.caritas-kissingen.de/beratung-und-hilfe/allgemeiner-sozialer-beratungsdienst</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q39" t="b">
+      <c r="P39" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3826,35 +3630,30 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 691-0</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>09521 691-0</t>
+          <t>caritas@caritas-hassberge.de</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>caritas@caritas-hassberge.de</t>
+          <t>http://www.caritas-hassberge.de/ich-brauche-hilfe/beratung/sozialberatung-allgemein</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>http://www.caritas-hassberge.de/ich-brauche-hilfe/beratung/sozialberatung-allgemein</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q40" t="b">
+      <c r="P40" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3911,35 +3710,30 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09321 2203-0</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>09321 2203-0</t>
+          <t>info@caritas-kitzingen.de</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>info@caritas-kitzingen.de</t>
+          <t>https://www.caritas-kitzingen.de/ich-brauche-hilfe/soziale-dienste/allgemeiner-sozialer-beratungsdienst</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>https://www.caritas-kitzingen.de/ich-brauche-hilfe/soziale-dienste/allgemeiner-sozialer-beratungsdienst</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q41" t="b">
+      <c r="P41" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3996,35 +3790,30 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09352 8431-19</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>09352 8431-19</t>
+          <t>geschaeftsstelle@caritas-msp.de</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>geschaeftsstelle@caritas-msp.de</t>
+          <t>https://www.caritas-msp.de/hilfe-und-beratung/allgemeiner-beratungsdienst</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>https://www.caritas-msp.de/hilfe-und-beratung/allgemeiner-beratungsdienst</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q42" t="b">
+      <c r="P42" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4081,35 +3870,30 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09371 9789-45</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>09371 9789-45</t>
+          <t>info@caritas-mil.de</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>info@caritas-mil.de</t>
+          <t>https://caritas-mil.de/elementor-8/beratung-unterstuetzung/</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>https://caritas-mil.de/elementor-8/beratung-unterstuetzung/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q43" t="b">
+      <c r="P43" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4166,35 +3950,30 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721/7158-30</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>09721/7158-30</t>
+          <t>asbd@caritas-schweinfurt.de</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>asbd@caritas-schweinfurt.de</t>
+          <t>http://caritas-sw.de/asbd/</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>http://caritas-sw.de/asbd/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q44" t="b">
+      <c r="P44" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4251,35 +4030,30 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09771 6116-0</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>09771 6116-0</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.caritas-rhoengrabfeld.de/ich-brauche-hilfe/allgemeiner-sozialer-beratungsdienst</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>http://www.caritas-rhoengrabfeld.de/ich-brauche-hilfe/allgemeiner-sozialer-beratungsdienst</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/allgemeine-sozialberatung/</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
           <t>contact_person, email</t>
         </is>
       </c>
-      <c r="Q45" t="b">
+      <c r="P45" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4336,35 +4110,30 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/fachambulanz-fuer-sexualstraftaeter/</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/fachambulanz-fuer-sexualstraftaeter/</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
-        <is>
           <t>organisation, website, contact_person</t>
         </is>
       </c>
-      <c r="Q46" t="b">
+      <c r="P46" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4421,35 +4190,30 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 571717</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0931 571717</t>
+          <t>info@fachstelle-suizidberatung.de</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>info@fachstelle-suizidberatung.de</t>
+          <t>http://www.fachstelle-suizidberatung.de</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>http://www.fachstelle-suizidberatung.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/krisenhilfe-telefonseelsorge-und-suizidpraevention/</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/krisenhilfe-telefonseelsorge-und-suizidpraevention/</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
           <t>organisation, contact_person</t>
         </is>
       </c>
-      <c r="Q47" t="b">
+      <c r="P47" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4506,35 +4270,30 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 322413</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0931 322413</t>
+          <t>info@christophorus.com</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>info@christophorus.com</t>
+          <t>http://www.christophorus-wuerzburg.de</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>http://www.christophorus-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q48" t="b">
+      <c r="P48" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4591,35 +4350,30 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09371 978957</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>09371 978957</t>
+          <t>schuldnerberatung@caritas-mil.de</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>schuldnerberatung@caritas-mil.de</t>
+          <t>https://caritas-mil.de/elementor-8/beratung-unterstuetzung/</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>https://caritas-mil.de/elementor-8/beratung-unterstuetzung/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q49" t="b">
+      <c r="P49" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4676,35 +4430,30 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 6910</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>09521 6910</t>
+          <t>sib@caritas-hassberge.de</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>sib@caritas-hassberge.de</t>
+          <t>https://www.caritas-hassberge.de/ich-brauche-hilfe/beratung/schulden-und-insolvenzberatung/</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>https://www.caritas-hassberge.de/ich-brauche-hilfe/beratung/schulden-und-insolvenzberatung/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q50" t="b">
+      <c r="P50" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4761,35 +4510,30 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 3301631</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>06021 3301631</t>
+          <t>schulderberatung@aschaffenburg.de</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>schulderberatung@aschaffenburg.de</t>
+          <t>https://www.aschaffenburg.de/Buerger-in-Aschaffenburg/Gesundheit-und-Soziales/Finanzielle-Hilfen-und-Notlagen/Schuldner--und-Insolvenzberatung/DE_index_3480.html</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>https://www.aschaffenburg.de/Buerger-in-Aschaffenburg/Gesundheit-und-Soziales/Finanzielle-Hilfen-und-Notlagen/Schuldner--und-Insolvenzberatung/DE_index_3480.html</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q51" t="b">
+      <c r="P51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4846,35 +4590,30 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 920 64 121</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>06021 920 64 121</t>
+          <t>schuldnerberatung@diakonie-aschaffenburg.de</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>schuldnerberatung@diakonie-aschaffenburg.de</t>
+          <t>https://diakonie-aschaffenburg.de/schuldnerberatung-insolvenzberatung</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>https://diakonie-aschaffenburg.de/schuldnerberatung-insolvenzberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q52" t="b">
+      <c r="P52" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4931,35 +4670,30 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0971 8012030</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0971 8012030</t>
+          <t>schuldnerberatung@kg.de</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>schuldnerberatung@kg.de</t>
+          <t>http://www.landkreis-badkissingen.de/buerger--politik/buergerservice/fachbereiche-und-abteilungen/jugend--soziales/soziales/schuldnerberatung/1122.Schuldner--und-Insolvenzberatung.html</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>http://www.landkreis-badkissingen.de/buerger--politik/buergerservice/fachbereiche-und-abteilungen/jugend--soziales/soziales/schuldnerberatung/1122.Schuldner--und-Insolvenzberatung.html</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Q53" t="b">
+      <c r="P53" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5016,35 +4750,30 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09771 6309715</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>09771 6309715</t>
+          <t>schuldnerberatung@diakonie-nes.de</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>schuldnerberatung@diakonie-nes.de</t>
+          <t>http://www.diakonie-nes.de/beratung/schuldner-und-insolvenzberatung</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>http://www.diakonie-nes.de/beratung/schuldner-und-insolvenzberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr">
-        <is>
           <t>organisation, contact_person</t>
         </is>
       </c>
-      <c r="Q54" t="b">
+      <c r="P54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5101,35 +4830,30 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09321 133840</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>09321 133840</t>
+          <t>schulderberatung@diakonie-kitzingen.de</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>schulderberatung@diakonie-kitzingen.de</t>
+          <t>https://www.diakonie-kitzingen.de/rat-hilfe/schuldner-und-insolvenzberatung</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>https://www.diakonie-kitzingen.de/rat-hilfe/schuldner-und-insolvenzberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q55" t="b">
+      <c r="P55" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5186,35 +4910,30 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721 7389590</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>09721 7389590</t>
+          <t>schuldnerberatung@kolping-schweinfurt.de</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>schuldnerberatung@kolping-schweinfurt.de</t>
+          <t>http://www.kolping-bildung-schweinfurt.de/angebote/schuldner-und-insolvenzberatung</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>http://www.kolping-bildung-schweinfurt.de/angebote/schuldner-und-insolvenzberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P56" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q56" t="b">
+      <c r="P56" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5271,35 +4990,30 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09353 7931136</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>09353 7931136</t>
+          <t>Hermann.Bulheller@Lramsp.de</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Hermann.Bulheller@Lramsp.de</t>
+          <t>https://www.main-spessart.de/buergerservice/sachgebiete-fachbereiche/index.html?detID=634&amp;catID=606</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>https://www.main-spessart.de/buergerservice/sachgebiete-fachbereiche/index.html?detID=634&amp;catID=606</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/schuldnerberatung/</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q57" t="b">
+      <c r="P57" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5356,35 +5070,30 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 55445</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>0931 55445</t>
+          <t>spdi.wuerzburg@tatenwerk.social</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>spdi.wuerzburg@tatenwerk.social</t>
+          <t>https://www.tatenwerk.social</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>https://www.tatenwerk.social</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
-        </is>
-      </c>
-      <c r="P58" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q58" t="b">
+      <c r="P58" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5441,35 +5150,30 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09351 2031</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>09351 2031</t>
+          <t>spdi.gemuenden@tatenwerk.social</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>spdi.gemuenden@tatenwerk.social</t>
+          <t>https://www.tatenwerk.social</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>https://www.tatenwerk.social</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q59" t="b">
+      <c r="P59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5526,35 +5230,30 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09391 917466</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>09391 917466</t>
+          <t>spdi.marktheidenfeld@tatenwerk.social</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>spdi.marktheidenfeld@tatenwerk.social</t>
+          <t>https://www.tatenwerk.social</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>https://www.tatenwerk.social</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
-        </is>
-      </c>
-      <c r="P60" t="inlineStr">
-        <is>
           <t>website, contact_person</t>
         </is>
       </c>
-      <c r="Q60" t="b">
+      <c r="P60" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5611,35 +5310,30 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 926550</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>09521 926550</t>
+          <t>spdi@caritas-hassberge.de</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>spdi@caritas-hassberge.de</t>
+          <t>https://www.caritas-hassberge.de</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>https://www.caritas-hassberge.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
-        </is>
-      </c>
-      <c r="P61" t="inlineStr">
-        <is>
           <t>organisation, website, contact_person</t>
         </is>
       </c>
-      <c r="Q61" t="b">
+      <c r="P61" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5696,35 +5390,30 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721 715 855</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>09721 715 855</t>
+          <t>spdi@caritas-schweinfurt.de</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>spdi@caritas-schweinfurt.de</t>
+          <t>https://www.caritas-schweinfurt.de</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>https://www.caritas-schweinfurt.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/sozialpsychiatrische-dienste/</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr">
-        <is>
           <t>organisation, website, contact_person</t>
         </is>
       </c>
-      <c r="Q62" t="b">
+      <c r="P62" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5781,35 +5470,30 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 392280</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>06021 392280</t>
+          <t>psb@caritas-aschaffenburg.de</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>psb@caritas-aschaffenburg.de</t>
+          <t>http://www.suchtberatung-aschaffenburg.de</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>http://www.suchtberatung-aschaffenburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P63" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q63" t="b">
+      <c r="P63" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5866,35 +5550,30 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0971 72469200</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0971 72469200</t>
+          <t>suchtberatung@caritas-kissingen.de</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>suchtberatung@caritas-kissingen.de</t>
+          <t>http://www.caritas-kissingen.de/beratung-und-hilfe/suchtberatung</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>http://www.caritas-kissingen.de/beratung-und-hilfe/suchtberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P64" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q64" t="b">
+      <c r="P64" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5951,35 +5630,30 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 926550</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>09521 926550</t>
+          <t>suchtberatung@caritas-hassberge.de</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>suchtberatung@caritas-hassberge.de</t>
+          <t>http://www.caritas-hassberge.de/ich-brauche-hilfe/beratung/suchtberatung</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>http://www.caritas-hassberge.de/ich-brauche-hilfe/beratung/suchtberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P65" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q65" t="b">
+      <c r="P65" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6036,35 +5710,30 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09321 22040</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>09321 22040</t>
+          <t>suchtberatung@caritas-kitzingen.de</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>suchtberatung@caritas-kitzingen.de</t>
+          <t>http://www.suchtberatung-kitzingen.org</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>http://www.suchtberatung-kitzingen.org</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P66" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q66" t="b">
+      <c r="P66" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6121,35 +5790,30 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09352 843121</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>09352 843121</t>
+          <t>psb@caritas-msp.de</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>psb@caritas-msp.de</t>
+          <t>http://www.caritas-msp.de/hilfe-und-beratung/suchtberatung/willkommen</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>http://www.caritas-msp.de/hilfe-und-beratung/suchtberatung/willkommen</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q67" t="b">
+      <c r="P67" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6206,35 +5870,30 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09371 978940</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>09371 978940</t>
+          <t>psb@caritas-mil.de</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>psb@caritas-mil.de</t>
+          <t>https://caritas-mil.de/beratung-unterstuetzung/#suchtberatung</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>https://caritas-mil.de/beratung-unterstuetzung/#suchtberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q68" t="b">
+      <c r="P68" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6291,35 +5950,30 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09771 61160</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>09771 61160</t>
+          <t>suchtberatung@caritas-nes.de</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>suchtberatung@caritas-nes.de</t>
+          <t>http://www.caritas-rhoengrabfeld.de/ich-brauche-hilfe/suchtberatung</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>http://www.caritas-rhoengrabfeld.de/ich-brauche-hilfe/suchtberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P69" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q69" t="b">
+      <c r="P69" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6376,35 +6030,30 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721 209550</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>09721 209550</t>
+          <t>suchtberatung@diakonie-schweinfurt.de</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>suchtberatung@diakonie-schweinfurt.de</t>
+          <t>http://www.diakonie-schweinfurt.de/rat-und-hilfe/sucht-und-abhaengigkeit</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>http://www.diakonie-schweinfurt.de/rat-und-hilfe/sucht-und-abhaengigkeit</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q70" t="b">
+      <c r="P70" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6461,35 +6110,30 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 38659180</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>0931 38659180</t>
+          <t>sucht@caritas-wuerzburg.org</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>sucht@caritas-wuerzburg.org</t>
+          <t>http://www.suchtberatung-wuerzburg.de</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>http://www.suchtberatung-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
           <t>organisation, contact_person</t>
         </is>
       </c>
-      <c r="Q71" t="b">
+      <c r="P71" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6546,35 +6190,30 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 59056</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>0931 59056</t>
+          <t>mail@drogenberatung-wuerzburg.de</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>mail@drogenberatung-wuerzburg.de</t>
+          <t>http://www.drogenberatung-wuerzburg.de</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>http://www.drogenberatung-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q72" t="b">
+      <c r="P72" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6631,35 +6270,30 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 35905220</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>0931 35905220</t>
+          <t>suchtberatung.wuerzburg@blaues-kreuz.de</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>suchtberatung.wuerzburg@blaues-kreuz.de</t>
+          <t>http://www.blaues-kreuz.de/bs-wuerzburg</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>http://www.blaues-kreuz.de/bs-wuerzburg</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q73" t="b">
+      <c r="P73" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6716,35 +6350,30 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 38658550</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>0931 38658550</t>
+          <t>info@kreuzbund-wuerzburg.de</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>info@kreuzbund-wuerzburg.de</t>
+          <t>http://www.kreuzbund-wuerzburg.de</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>http://www.kreuzbund-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/suchtberatung/</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q74" t="b">
+      <c r="P74" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6801,35 +6430,30 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>06021 392-121</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>06021 392-121</t>
+          <t>w.katholing@caritas-aschaffenburg.de</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>w.katholing@caritas-aschaffenburg.de</t>
+          <t>https://www.caritas-aschaffenburg.de/sie-suchen-hilfe/fl%C3%BCchtlings-und-integrationsberatung</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>https://www.caritas-aschaffenburg.de/sie-suchen-hilfe/fl%C3%BCchtlings-und-integrationsberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q75" t="b">
+      <c r="P75" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6886,35 +6510,30 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0971 7246-9200</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>0971 7246-9200</t>
+          <t>j.ort@caritas-kissingen.de</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>j.ort@caritas-kissingen.de</t>
+          <t>https://www.caritas-kissingen.de/beratung-und-hilfe/asyl-und-migration</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>https://www.caritas-kissingen.de/beratung-und-hilfe/asyl-und-migration</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q76" t="b">
+      <c r="P76" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6971,35 +6590,30 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09771 6116-25</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>09771 6116-25</t>
+          <t>silvia.baumbach@caritas-nes.de</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>silvia.baumbach@caritas-nes.de</t>
+          <t>https://www.caritas-rhoengrabfeld.de/ich-brauche-hilfe/fl%C3%BCchtlings-und-integrationsberatung</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>https://www.caritas-rhoengrabfeld.de/ich-brauche-hilfe/fl%C3%BCchtlings-und-integrationsberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q77" t="b">
+      <c r="P77" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7056,35 +6670,30 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09521 952974-0</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>09521 952974-0</t>
+          <t>asyl@caritas-hassberge.de</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>asyl@caritas-hassberge.de</t>
+          <t>http://www.asylberatung.caritas-hassberge.de</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>http://www.asylberatung.caritas-hassberge.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q78" t="b">
+      <c r="P78" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7141,35 +6750,30 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09371 9789-45</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>09371 9789-45</t>
+          <t>w-haertel@caritas-mil.de</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>w-haertel@caritas-mil.de</t>
+          <t>https://www.caritas-mil.de/beratung-und-unterst%C3%BCtzung/fluechtlings-und-integrationsberatung</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>https://www.caritas-mil.de/beratung-und-unterst%C3%BCtzung/fluechtlings-und-integrationsberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P79" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q79" t="b">
+      <c r="P79" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7226,35 +6830,30 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09321 220-30</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>09321 220-30</t>
+          <t>info@caritas-kitzingen.de</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>info@caritas-kitzingen.de</t>
+          <t>https://www.caritas-kitzingen.de/ich-brauche-hilfe/fluchtlings-und-integrationsberatung/</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>https://www.caritas-kitzingen.de/ich-brauche-hilfe/fluchtlings-und-integrationsberatung/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q80" t="b">
+      <c r="P80" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7311,35 +6910,30 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09721 6537-304</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>09721 6537-304</t>
+          <t>blauth@erstaufnahme-sw.de</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>blauth@erstaufnahme-sw.de</t>
+          <t>http://www.caritas-sw.de/</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>http://www.caritas-sw.de/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P81" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q81" t="b">
+      <c r="P81" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7396,35 +6990,30 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>09352 8431-17</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>09352 8431-17</t>
+          <t>fluechtlingsberatung@caritas-msp.de</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>fluechtlingsberatung@caritas-msp.de</t>
+          <t>https://www.caritas-msp.de/hilfe-und-beratung/fl%C3%BCchtlings-und-integrationsberatung</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>https://www.caritas-msp.de/hilfe-und-beratung/fl%C3%BCchtlings-und-integrationsberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P82" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q82" t="b">
+      <c r="P82" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7481,35 +7070,30 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-58170</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>0931 386-58170</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P83" t="inlineStr">
-        <is>
           <t>email, contact_person</t>
         </is>
       </c>
-      <c r="Q83" t="b">
+      <c r="P83" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7566,35 +7150,30 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66782</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>0931 386-66782</t>
+          <t>info@zrb-westbayern.de</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>info@zrb-westbayern.de</t>
+          <t>http://zrb-nordbayern.de/</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>http://zrb-nordbayern.de/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/adressen-migrationsdienste/</t>
-        </is>
-      </c>
-      <c r="P84" t="inlineStr">
-        <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="Q84" t="b">
+      <c r="P84" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7651,17 +7230,17 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 38658152</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>0931 38658152</t>
+          <t>rainer.jaeckel@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>rainer.jaeckel@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -7671,15 +7250,10 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
-        </is>
-      </c>
-      <c r="P85" t="inlineStr">
-        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="Q85" t="b">
+      <c r="P85" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7736,17 +7310,17 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -7756,15 +7330,10 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
-        </is>
-      </c>
-      <c r="P86" t="inlineStr">
-        <is>
           <t>phone, email, website, contact_person</t>
         </is>
       </c>
-      <c r="Q86" t="b">
+      <c r="P86" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7821,17 +7390,17 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 467659-01</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>0931 467659-01</t>
+          <t>nicole.goessl@caritas-wuerzburg.de; romina.gulyas@caritas-wuerzburg.de; sebastian.neumeyer@caritas-wuerzburg.de; sergo.titali@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>nicole.goessl@caritas-wuerzburg.de; romina.gulyas@caritas-wuerzburg.de; sebastian.neumeyer@caritas-wuerzburg.de; sergo.titali@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -7841,15 +7410,10 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
           <t>organisation, website</t>
         </is>
       </c>
-      <c r="Q87" t="b">
+      <c r="P87" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7906,35 +7470,30 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-58150</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>0931 386-58150</t>
+          <t>nicole.goessl@caritas-wuerzburg.de; romina.gulyas@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>nicole.goessl@caritas-wuerzburg.de; romina.gulyas@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/beratung-in-wuerzburg/</t>
-        </is>
-      </c>
-      <c r="P88" t="inlineStr">
-        <is>
           <t>organisation, website</t>
         </is>
       </c>
-      <c r="Q88" t="b">
+      <c r="P88" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7991,17 +7550,17 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/besuchsdienste/</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -8011,15 +7570,10 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/besuchsdienste/</t>
-        </is>
-      </c>
-      <c r="P89" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q89" t="b">
+      <c r="P89" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8076,17 +7630,17 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/familienpflege/</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -8096,15 +7650,10 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/familienpflege/</t>
-        </is>
-      </c>
-      <c r="P90" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q90" t="b">
+      <c r="P90" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8161,17 +7710,17 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/jugendhilfe/</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -8181,15 +7730,10 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/jugendhilfe/</t>
-        </is>
-      </c>
-      <c r="P91" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q91" t="b">
+      <c r="P91" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8246,35 +7790,30 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://caritas-kitzingen.de/ich-will-helfen/nachbarschaftshilfe</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>https://caritas-kitzingen.de/ich-will-helfen/nachbarschaftshilfe</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/nachbarschaftshilfe/</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/nachbarschaftshilfe/</t>
-        </is>
-      </c>
-      <c r="P92" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q92" t="b">
+      <c r="P92" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8331,35 +7870,30 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.skf-aschaffenburg.de</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>http://www.skf-aschaffenburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/schwangerschaftsberatung/</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/schwangerschaftsberatung/</t>
-        </is>
-      </c>
-      <c r="P93" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q93" t="b">
+      <c r="P93" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8416,35 +7950,30 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.skf-wue.de/index.php?id=185</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>http://www.skf-wue.de/index.php?id=185</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/schwangerschaftsberatung/</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/schwangerschaftsberatung/</t>
-        </is>
-      </c>
-      <c r="P94" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q94" t="b">
+      <c r="P94" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8501,35 +8030,30 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.skf-schweinfurt.de/hilfe-beratung/schwangerschaftsberatung</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>https://www.skf-schweinfurt.de/hilfe-beratung/schwangerschaftsberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/schwangerschaftsberatung/</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/familie/schwangerschaftsberatung/</t>
-        </is>
-      </c>
-      <c r="P95" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q95" t="b">
+      <c r="P95" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8586,17 +8110,17 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/essstoerungen/</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -8606,15 +8130,10 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/essstoerungen/</t>
-        </is>
-      </c>
-      <c r="P96" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q96" t="b">
+      <c r="P96" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8671,17 +8190,17 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendwohnen/</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -8691,15 +8210,10 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/jugendwohnen/</t>
-        </is>
-      </c>
-      <c r="P97" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q97" t="b">
+      <c r="P97" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8756,17 +8270,17 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/junge-eltern-und-beruf/</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -8776,15 +8290,10 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/jugend/junge-eltern-und-beruf/</t>
-        </is>
-      </c>
-      <c r="P98" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q98" t="b">
+      <c r="P98" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8841,35 +8350,30 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.skf-wue.de</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>http://www.skf-wue.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
-        </is>
-      </c>
-      <c r="P99" t="inlineStr">
-        <is>
           <t>street, phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q99" t="b">
+      <c r="P99" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8926,35 +8430,30 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.skf-schweinfurt.de</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>http://www.skf-schweinfurt.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
-        </is>
-      </c>
-      <c r="P100" t="inlineStr">
-        <is>
           <t>street, phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q100" t="b">
+      <c r="P100" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9011,35 +8510,30 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.skf-aschaffenburg.de</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>http://www.skf-aschaffenburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr">
-        <is>
           <t>street, phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q101" t="b">
+      <c r="P101" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9096,35 +8590,30 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.invia-wuerzburg.de</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>http://www.invia-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
-        </is>
-      </c>
-      <c r="P102" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q102" t="b">
+      <c r="P102" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9181,35 +8670,30 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>http://www.invia-aschaffenburg.de</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>http://www.invia-aschaffenburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hilfen-fuer-frauen-1/</t>
-        </is>
-      </c>
-      <c r="P103" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q103" t="b">
+      <c r="P103" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9266,17 +8750,17 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hivaids/</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -9286,15 +8770,10 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/hivaids/</t>
-        </is>
-      </c>
-      <c r="P104" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q104" t="b">
+      <c r="P104" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9351,17 +8830,17 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/straffaelligenhilfe/</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -9371,15 +8850,10 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/straffaelligenhilfe/</t>
-        </is>
-      </c>
-      <c r="P105" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q105" t="b">
+      <c r="P105" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9436,35 +8910,30 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.bahnhofsmission-wuerzburg.de/</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>https://www.bahnhofsmission-wuerzburg.de/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
-        </is>
-      </c>
-      <c r="P106" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q106" t="b">
+      <c r="P106" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9521,35 +8990,30 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.invia-wuerzburg.de/leistungen-und-einrichtungen/</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>https://www.invia-wuerzburg.de/leistungen-und-einrichtungen/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
-        </is>
-      </c>
-      <c r="P107" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q107" t="b">
+      <c r="P107" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9606,35 +9070,30 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://www.bahnhofsmission-aschaffenburg.de/</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>https://www.bahnhofsmission-aschaffenburg.de/</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
-        </is>
-      </c>
-      <c r="P108" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q108" t="b">
+      <c r="P108" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9691,35 +9150,30 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>0931 386-66 700 (Zentrale Caritas Diözese)</t>
+          <t>info@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>info@caritas-wuerzburg.de</t>
+          <t>https://caritas-mil.de/beratung-unterstuetzung/#wohnungslosenberatung</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>https://caritas-mil.de/beratung-unterstuetzung/#wohnungslosenberatung</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-in-krisensituationen/wohnsitzlosigkeit/</t>
-        </is>
-      </c>
-      <c r="P109" t="inlineStr">
-        <is>
           <t>street, contact_person, phone, email</t>
         </is>
       </c>
-      <c r="Q109" t="b">
+      <c r="P109" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9776,17 +9230,17 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-mit-behinderung/foerderschulen/</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -9796,15 +9250,10 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/menschen-mit-behinderung/foerderschulen/</t>
-        </is>
-      </c>
-      <c r="P110" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q110" t="b">
+      <c r="P110" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9861,17 +9310,17 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/rueckkehrberatung/</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -9881,15 +9330,10 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/migrationasyl/rueckkehrberatung/</t>
-        </is>
-      </c>
-      <c r="P111" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q111" t="b">
+      <c r="P111" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9946,17 +9390,17 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/ambulante-pflege/</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -9966,15 +9410,10 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/ambulante-pflege/</t>
-        </is>
-      </c>
-      <c r="P112" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q112" t="b">
+      <c r="P112" t="b">
         <v>1</v>
       </c>
     </row>
@@ -10031,17 +9470,17 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/ambulante-wohngemeinschaften/</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -10051,15 +9490,10 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/ambulante-wohngemeinschaften/</t>
-        </is>
-      </c>
-      <c r="P113" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q113" t="b">
+      <c r="P113" t="b">
         <v>1</v>
       </c>
     </row>
@@ -10116,17 +9550,17 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/palliativ-ethik-und-hospizarbeit/</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -10136,15 +9570,10 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/palliativ-ethik-und-hospizarbeit/</t>
-        </is>
-      </c>
-      <c r="P114" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q114" t="b">
+      <c r="P114" t="b">
         <v>1</v>
       </c>
     </row>
@@ -10201,17 +9630,17 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/teilstationaere-altenhilfe/</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -10221,15 +9650,10 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/teilstationaere-altenhilfe/</t>
-        </is>
-      </c>
-      <c r="P115" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q115" t="b">
+      <c r="P115" t="b">
         <v>1</v>
       </c>
     </row>
@@ -10286,17 +9710,17 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>0931 386-66500</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>0931 386-66500</t>
+          <t>fachambulanz@caritas-wuerzburg.de</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>fachambulanz@caritas-wuerzburg.de</t>
+          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/vollstationaere-pflege/</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -10306,20 +9730,15 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>https://www.caritas-wuerzburg.de/hilfe-beratung/senioren/altenhilfe/vollstationaere-pflege/</t>
-        </is>
-      </c>
-      <c r="P116" t="inlineStr">
-        <is>
           <t>phone, email, contact_person</t>
         </is>
       </c>
-      <c r="Q116" t="b">
+      <c r="P116" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q116"/>
+  <autoFilter ref="A1:P116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>